<commit_message>
Align Qwen 910B offload and MemCache sizing
</commit_message>
<xml_diff>
--- a/wings_control/docs/DAY0/qwen优化参数适配基准.xlsx
+++ b/wings_control/docs/DAY0/qwen优化参数适配基准.xlsx
@@ -1102,7 +1102,7 @@
           <t>否</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
           <t>否</t>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>rebuilt from qwen model collection workbook and aligned with adaptation design baseline</t>
+          <t>rebuilt from qwen model collection workbook and aligned with adaptation design baseline; current adaptation policy: Qwen3.5/3.6 on 910B keeps MTP but disables MemCache/offload</t>
         </is>
       </c>
     </row>
@@ -2494,19 +2494,15 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>MTP+MemCache</t>
+          <t>MTP-only</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>50051/50061</t>
-        </is>
-      </c>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="inlineStr">
         <is>
           <t>否</t>
@@ -2651,7 +2647,7 @@
       <c r="AK9" s="2" t="inlineStr"/>
       <c r="AL9" s="2" t="inlineStr">
         <is>
-          <t>rebuilt from qwen model collection workbook and aligned with adaptation design baseline</t>
+          <t>rebuilt from qwen model collection workbook and aligned with adaptation design baseline; current adaptation policy: Qwen3.5/3.6 on 910B keeps MTP but disables MemCache/offload</t>
         </is>
       </c>
     </row>
@@ -3096,19 +3092,15 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>MTP+MemCache</t>
+          <t>MTP-only</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>50051/50061</t>
-        </is>
-      </c>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
           <t>是</t>
@@ -3254,7 +3246,7 @@
       <c r="AK12" s="2" t="inlineStr"/>
       <c r="AL12" s="2" t="inlineStr">
         <is>
-          <t>rebuilt from qwen model collection workbook and aligned with adaptation design baseline</t>
+          <t>rebuilt from qwen model collection workbook and aligned with adaptation design baseline; current adaptation policy: Qwen3.5/3.6 on 910B keeps MTP but disables MemCache/offload</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4479,6 +4471,18 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>qwen_910b_offload_policy</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Qwen3.5/3.6 910B场景保留MTP，统一禁用MemCache/offload；910C策略不变</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>